<commit_message>
Start 23 Sep: add item 1, black Krizia jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6218,8 +6218,47 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>Krizia Jacket (brand to confirm)</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>Black, tailored women's fit</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr"/>
+      <c r="G115" s="7" t="inlineStr"/>
+      <c r="H115" s="7" t="inlineStr"/>
+      <c r="I115" s="8" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="J115" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K115" s="9" t="n">
+        <v>46288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K114"/>
+  <autoFilter ref="A1:K115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set condition on 23 Sep item 1
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -6243,7 +6243,11 @@
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr"/>
-      <c r="G115" s="7" t="inlineStr"/>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
       <c r="H115" s="7" t="inlineStr"/>
       <c r="I115" s="8" t="n">
         <v>44.99</v>

</xml_diff>

<commit_message>
Add 23 Sep item 2: Fay gilet
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6261,8 +6261,51 @@
         <v>46288</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Fay Gilet (brand to confirm)</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr"/>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>Medium Men's</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr"/>
+      <c r="I116" s="4" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K116" s="5" t="n">
+        <v>46288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K115"/>
+  <autoFilter ref="A1:K116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 23 Sep item 3: Dolce & Gabbana jacket with fur collar
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6304,8 +6304,56 @@
         <v>46288</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>Dolce &amp; Gabbana Jacket</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Fur-lined collar
+Very small red imperfection on the front left, by the pocket near the logo (see images)</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Very small red imperfection on the front left, by the pocket near the logo (see images)</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr"/>
+      <c r="I117" s="4" t="n">
+        <v>89.98999999999999</v>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="n">
+        <v>46288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K116"/>
+  <autoFilter ref="A1:K117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 23 Sep item 4: Belstaff jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6352,8 +6352,51 @@
         <v>46288</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Belstaff Jacket</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr"/>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>XL or XXL (unconfirmed)</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr"/>
+      <c r="I118" s="4" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="n">
+        <v>46288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K117"/>
+  <autoFilter ref="A1:K118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 23 Sep item 5: Moncler jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6395,8 +6395,51 @@
         <v>46288</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Moncler Jacket</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr"/>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>Large or XL (unconfirmed - check numeric label)</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr"/>
+      <c r="I119" s="4" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="n">
+        <v>46288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K118"/>
+  <autoFilter ref="A1:K119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 28 Sep item 9, export the day, rebuild the workbook
A Large Lacoste polo at 16.00 rules out size as the explanation for the
12.99 one, leaving the "very good vintage" grading as the best
remaining candidate.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$149</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6248,7 +6248,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="H115" s="7" t="inlineStr"/>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
       <c r="I115" s="8" t="n">
         <v>44.99</v>
       </c>
@@ -6291,7 +6295,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="H116" s="3" t="inlineStr"/>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
       <c r="I116" s="4" t="n">
         <v>39.99</v>
       </c>
@@ -6339,7 +6347,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="H117" s="3" t="inlineStr"/>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
       <c r="I117" s="4" t="n">
         <v>89.98999999999999</v>
       </c>
@@ -6382,7 +6394,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="H118" s="3" t="inlineStr"/>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
       <c r="I118" s="4" t="n">
         <v>79.98999999999999</v>
       </c>
@@ -6425,7 +6441,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="H119" s="3" t="inlineStr"/>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
       <c r="I119" s="4" t="n">
         <v>129.99</v>
       </c>
@@ -6438,8 +6458,1321 @@
         <v>46288</v>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>Fay Trench Jacket (brand to confirm)</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>Single Fay hook-and-clasp fastening at the neck (not the four-hook 4 Ganci style)</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>XS Women's</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K120" s="5" t="n">
+        <v>46288</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B121" s="7" t="inlineStr"/>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>Les Copains Denim Jacket</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Green-toned denim</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>(see collar label)</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="J121" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K121" s="9" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Emanuel Ungaro Jacket</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>White women's jacket. Made in Italy.
+Small discrepancy on the front - minor and barely noticeable</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Small discrepancy on the front - minor and barely noticeable</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr"/>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K122" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Barbour Beaufort Waxed Jacket</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Brown waxed cotton (Rustic/Bark colourway). Beaufort model.</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>XL (unconfirmed - Barbour sizes by chest, check the C__/__CM label)</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>Trussardi Action Coat</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>Brown. Labelled real leather - appears suede or nubuck rather than smooth leather (material to confirm)</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>IT 50 (UK 40 chest / Large mens)</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="3" t="inlineStr"/>
+      <c r="K124" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>Hugo Boss Leather Jacket</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Leather with a removable interior liner</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr"/>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
+      <c r="K125" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>GFF Gianfranco Ferre Jacket</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr"/>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>IT 46 / USA 12 (approx UK 12-14 - vintage sizing runs small, confirm by measurement)</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr"/>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr"/>
+      <c r="K126" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B127" s="3" t="inlineStr"/>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Cacharel Cashmere Knitted Cardigan / Jacket</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Cashmere knitted cardigan-jacket</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>(no size label - needs measuring)</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr"/>
+      <c r="K127" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>Fur Jacket</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>Fur - confirm real or faux before listing (platform restrictions apply)</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr"/>
+      <c r="K128" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>Mizone Uomo Cardigan (brand to confirm)</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>Several discolourations</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Several discolourations</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr"/>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactory condition</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr"/>
+      <c r="K129" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Burberry Jacket</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>Label reads Burberry, not Burberrys - dates it post-1999</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>Taglia/Talla 54 (continental) - reads as men's XL / UK 44 chest. If genuinely women's it would be UK 22. Confirm by placket direction</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr"/>
+      <c r="K130" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B131" s="3" t="inlineStr"/>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Barbour Dress Tartan Jacket</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Barbour Dress Tartan (the house tartan, red/pink based)</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>SF3</t>
+        </is>
+      </c>
+      <c r="I131" s="4" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr"/>
+      <c r="K131" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Pal Zileri Sport Jacket</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr"/>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I132" s="4" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr"/>
+      <c r="K132" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B133" s="3" t="inlineStr"/>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Easy by Nazareno Gabrielli Jacket</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Navy with a teal lining. Zip-off sleeves and a button-off hood, so it converts to a gilet.
+Broken zip</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>Broken zip (confirm which - main front zip or a sleeve zip)</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr"/>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I133" s="4" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr"/>
+      <c r="K133" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B134" s="3" t="inlineStr"/>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Diesel Jacket</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>Butter yellow.
+A few discolouration marks, not very noticeable</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>A few discolouration marks, not very noticeable</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I134" s="4" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr"/>
+      <c r="K134" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Pierre Cardin Jacket</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Navy.
+The bottom part of the zip has snapped off, but the zip still works fine</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>Bottom part of the zip has snapped off - zip still works fine</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>102cm chest (40 inch / Large mens)</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I135" s="4" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr"/>
+      <c r="K135" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B136" s="3" t="inlineStr"/>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Belstaff Jacket</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr"/>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Jackets</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr"/>
+      <c r="K136" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B137" s="3" t="inlineStr"/>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>Green.
+A few tiny snag holes</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>A few tiny snag holes</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr"/>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I137" s="4" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr"/>
+      <c r="K137" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B138" s="3" t="inlineStr"/>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Cardigan</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>Blue. No inside label.</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G138" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H138" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I138" s="4" t="inlineStr"/>
+      <c r="J138" s="3" t="inlineStr"/>
+      <c r="K138" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B139" s="3" t="inlineStr"/>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Cardigan</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Beige. No inside labels.
+2 small stains on the front of the sleeve</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>2 small stains on the front of the sleeve</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr"/>
+      <c r="G139" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H139" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I139" s="4" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr"/>
+      <c r="K139" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B140" s="3" t="inlineStr"/>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Jacket</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Charcoal grey. No inside label.</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G140" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H140" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I140" s="4" t="inlineStr"/>
+      <c r="J140" s="3" t="inlineStr"/>
+      <c r="K140" s="5" t="n">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Hoodie</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G141" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H141" s="7" t="inlineStr">
+        <is>
+          <t>VWM - Hoodies/Sweatshirts</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="J141" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>Izod Lacoste Cardigan</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr"/>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I142" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="J142" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K142" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>Izod Lacoste Cardigan</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Light blue.
+The fourth button down is chipped - only half of it remains</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>Fourth button down is chipped - only half of it remains</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I143" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="J143" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K143" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Hugo Boss Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Dark grey</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="inlineStr"/>
+      <c r="I144" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J144" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K144" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B145" s="3" t="inlineStr"/>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Krizia Jeans T-Shirt</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>Small (a bit of a big fit)</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Summer Mix</t>
+        </is>
+      </c>
+      <c r="I145" s="4" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Hugo Boss Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr"/>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Summer Mix</t>
+        </is>
+      </c>
+      <c r="I146" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J146" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Lululemon Full-Zip Jacket (product type to confirm)</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Brown. Full-length zip with a long funnel neck.</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr"/>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="I147" s="4" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Prada Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>A few minor marks on the front</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>A few minor marks on the front</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>SF - Men's Summer Designer Mix</t>
+        </is>
+      </c>
+      <c r="I148" s="4" t="inlineStr"/>
+      <c r="J148" s="3" t="inlineStr"/>
+      <c r="K148" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr"/>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="I149" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K119"/>
+  <autoFilter ref="A1:K149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Re-export the full 28 Sep batch and rebuild the workbook
Twenty-one items, twelve priced at 257.96, nine for the photo chat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7771,8 +7771,547 @@
         <v>46293</v>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>38 (French/EU - approx UK 10)</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I150" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Izod Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr"/>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I151" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="J151" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K151" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B152" s="3" t="inlineStr"/>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>Jeans Les Copains Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Multicoloured</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>IV (Roman numeral - Large or XL, confirm by measurement)</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr"/>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Summer Mix</t>
+        </is>
+      </c>
+      <c r="I152" s="4" t="inlineStr"/>
+      <c r="J152" s="3" t="inlineStr"/>
+      <c r="K152" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B153" s="3" t="inlineStr"/>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Blue and black striped</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>3XL (US)</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I153" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>Polo Shirt (brand not stated)</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Red/pink</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>46 (continental - UK 36in chest / Small)</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - Summer Mix</t>
+        </is>
+      </c>
+      <c r="I154" s="4" t="inlineStr"/>
+      <c r="J154" s="3" t="inlineStr"/>
+      <c r="K154" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Argyle Cardigan</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Cream with a grey diamond (argyle) pattern on the front</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I155" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>Chaps Ralph Lauren Anorak (confirm pullover or full-zip)</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Khaki/green.
+Slight nicks to the badge on the front (see images). Interior a bit worn but nothing major.</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>Slight nicks to the badge on the front (see images). Interior a bit worn but nothing major.</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr"/>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="I156" s="4" t="inlineStr"/>
+      <c r="J156" s="3" t="inlineStr"/>
+      <c r="K156" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B157" s="3" t="inlineStr"/>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Tommy Hilfiger Polo Shirt</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Light blue.
+A few white discrepancies on the front</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>A few white discrepancies on the front</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr"/>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>SF Fripe - RL Tommy Lacoste Mix</t>
+        </is>
+      </c>
+      <c r="I157" s="4" t="inlineStr"/>
+      <c r="J157" s="3" t="inlineStr"/>
+      <c r="K157" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Nike Jacket</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr"/>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="I158" s="4" t="inlineStr"/>
+      <c r="J158" s="3" t="inlineStr"/>
+      <c r="K158" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B159" s="3" t="inlineStr"/>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Club Cardigan</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Red.
+Slight dark discolouration at the bottom, near the buttons (see images)</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>Slight dark discolouration at the bottom, near the buttons (see images)</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Good vintage condition</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I159" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Tommy Hilfiger Jacket</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr"/>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>Large (labelled Small but fits large - confirm by measurement)</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="3" t="inlineStr"/>
+      <c r="K160" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Nike Windbreaker</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Yellow and navy</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>Medium (oversized fit)</t>
+        </is>
+      </c>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="I161" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="J161" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="n">
+        <v>46293</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K149"/>
+  <autoFilter ref="A1:K161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>